<commit_message>
Update .xlsx - Alternative lure for Old/New task
Added condition column to distinguish lure subtypes in Old/New task
fixed a warning about a typo on ObScene file name
</commit_message>
<xml_diff>
--- a/Exemplo_encode.xlsx
+++ b/Exemplo_encode.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vera/Documents/GitHub/SEED/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD706F4-8F12-EB4E-9BD6-FC831B28A65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42CBDF76-3231-B74F-AB07-9486D743FD66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2240" yWindow="3600" windowWidth="23480" windowHeight="10980" xr2:uid="{BC1145FC-44B2-8E4A-B352-2463BCCE776C}"/>
   </bookViews>
@@ -561,7 +561,7 @@
   <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="29.6640625" customWidth="1"/>
+    <col min="2" max="2" width="35.6640625" customWidth="1"/>
     <col min="4" max="4" width="30.33203125" customWidth="1"/>
     <col min="5" max="6" width="14.5" customWidth="1"/>
     <col min="7" max="7" width="15.1640625" customWidth="1"/>

</xml_diff>